<commit_message>
Add missing requirement numbers
</commit_message>
<xml_diff>
--- a/input/requirements/Procedure.xlsx
+++ b/input/requirements/Procedure.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30203"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nictiznl.sharepoint.com/sites/Zib-transitiecommunity/Gedeelde documenten/Architectuur/Werkgroepen ZIBS 2.0 Implementatie/Bouwblokken/Verrichting - Spirit/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\edelman_nict1\IGs\GBB-IG\input\requirements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{491BA9B5-C372-4BED-9655-F4102442FCE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41642281-4408-4428-AC78-DE7A4991C766}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-72" yWindow="2316" windowWidth="29016" windowHeight="13500" firstSheet="2" activeTab="2" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="2" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
   </bookViews>
   <sheets>
     <sheet name="Uitleg" sheetId="5" r:id="rId1"/>
@@ -370,7 +370,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="371">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="373">
   <si>
     <t>Veld</t>
   </si>
@@ -1487,13 +1487,19 @@
   </si>
   <si>
     <t>Er is op dit moment nog geen input binnengekomen van team Topgun, waardoor het gebruik en de wensen omtrent verrichting niet meegenomen zijn in deze eerste ontwikkelfase.</t>
+  </si>
+  <si>
+    <t>4.2.1</t>
+  </si>
+  <si>
+    <t>4.2.2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1634,7 +1640,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2750,12 +2756,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F1013F7-63B2-4F83-92B0-1C8153859891}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="218.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="15" customHeight="1">
+    <row r="1" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3"/>
     </row>
   </sheetData>
@@ -2767,7 +2773,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CC1E3B3-D087-4A2B-920B-9BA971FAD64B}">
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
     <col min="2" max="2" width="32.7109375" customWidth="1"/>
@@ -2775,10 +2781,10 @@
     <col min="4" max="4" width="99.85546875" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="190.5" customHeight="1">
+    <row r="1" spans="1:4" ht="190.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3"/>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -2786,7 +2792,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="28.9">
+    <row r="3" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -2797,7 +2803,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="100.9">
+    <row r="4" spans="1:4" ht="105" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -2808,7 +2814,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="57.6">
+    <row r="5" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -2819,7 +2825,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="57.6">
+    <row r="6" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -2830,7 +2836,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="28.9">
+    <row r="7" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -2841,7 +2847,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="28.9">
+    <row r="8" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -2852,7 +2858,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="57.6">
+    <row r="9" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -2866,7 +2872,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="57.6">
+    <row r="10" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>24</v>
       </c>
@@ -2890,7 +2896,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7034CDAF-2A08-4BE8-92C3-F4E7A6F24E1B}">
   <dimension ref="A1:K75"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="22.42578125" style="4" customWidth="1"/>
     <col min="3" max="3" width="14.85546875" style="4" customWidth="1"/>
@@ -2903,8 +2909,8 @@
     <col min="11" max="11" width="19.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="88.5" customHeight="1"/>
-    <row r="2" spans="1:11" ht="28.9">
+    <row r="1" spans="1:11" ht="88.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>28</v>
       </c>
@@ -2937,7 +2943,7 @@
       </c>
       <c r="K2" s="2"/>
     </row>
-    <row r="3" spans="1:11" ht="28.9">
+    <row r="3" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="6">
         <v>1</v>
       </c>
@@ -2960,7 +2966,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="43.15">
+    <row r="4" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>43</v>
       </c>
@@ -2987,7 +2993,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="43.15">
+    <row r="5" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>48</v>
       </c>
@@ -3014,7 +3020,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="28.9">
+    <row r="6" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>52</v>
       </c>
@@ -3041,7 +3047,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="43.15">
+    <row r="7" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>58</v>
       </c>
@@ -3068,7 +3074,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="28.9">
+    <row r="8" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>65</v>
       </c>
@@ -3093,7 +3099,7 @@
       </c>
       <c r="J8" s="3"/>
     </row>
-    <row r="9" spans="1:11" ht="28.9">
+    <row r="9" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>71</v>
       </c>
@@ -3118,7 +3124,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="28.9">
+    <row r="10" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>77</v>
       </c>
@@ -3141,7 +3147,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="15" customHeight="1">
+    <row r="11" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>82</v>
       </c>
@@ -3173,7 +3179,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="28.9">
+    <row r="12" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="4">
         <v>2</v>
       </c>
@@ -3193,7 +3199,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="14.45">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
         <v>96</v>
       </c>
@@ -3213,7 +3219,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="14.45">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
         <v>100</v>
       </c>
@@ -3233,7 +3239,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="14.45">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
         <v>104</v>
       </c>
@@ -3253,7 +3259,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="14.45">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="4">
         <v>3</v>
       </c>
@@ -3267,7 +3273,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="14.45">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
         <v>110</v>
       </c>
@@ -3294,7 +3300,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="14.45">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>117</v>
       </c>
@@ -3317,7 +3323,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="14.45">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>123</v>
       </c>
@@ -3343,7 +3349,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="14.45">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
         <v>129</v>
       </c>
@@ -3369,7 +3375,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="57.6">
+    <row r="21" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A21" s="6">
         <v>4</v>
       </c>
@@ -3392,7 +3398,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="28.9">
+    <row r="22" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>137</v>
       </c>
@@ -3417,7 +3423,7 @@
       </c>
       <c r="J22" s="3"/>
     </row>
-    <row r="23" spans="1:10" ht="28.9">
+    <row r="23" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>143</v>
       </c>
@@ -3440,7 +3446,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="28.9">
+    <row r="24" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>146</v>
       </c>
@@ -3463,7 +3469,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="28.9">
+    <row r="25" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>149</v>
       </c>
@@ -3486,7 +3492,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="28.9">
+    <row r="26" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
         <v>153</v>
       </c>
@@ -3509,7 +3515,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="28.9">
+    <row r="27" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
         <v>157</v>
       </c>
@@ -3532,7 +3538,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="28.9">
+    <row r="28" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
         <v>161</v>
       </c>
@@ -3555,7 +3561,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="28.9">
+    <row r="29" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
         <v>164</v>
       </c>
@@ -3578,7 +3584,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="28.9">
+    <row r="30" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
         <v>169</v>
       </c>
@@ -3601,7 +3607,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="28.9">
+    <row r="31" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
         <v>173</v>
       </c>
@@ -3624,7 +3630,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="28.9">
+    <row r="32" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
         <v>177</v>
       </c>
@@ -3647,7 +3653,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="28.9">
+    <row r="33" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
         <v>181</v>
       </c>
@@ -3670,7 +3676,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="28.9">
+    <row r="34" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
         <v>185</v>
       </c>
@@ -3693,7 +3699,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="35" spans="1:10" ht="28.9">
+    <row r="35" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
         <v>189</v>
       </c>
@@ -3716,7 +3722,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="36" spans="1:10" ht="28.9">
+    <row r="36" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
         <v>193</v>
       </c>
@@ -3739,7 +3745,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="37" spans="1:10" ht="28.9">
+    <row r="37" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
         <v>197</v>
       </c>
@@ -3762,7 +3768,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="38" spans="1:10" ht="43.15">
+    <row r="38" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
         <v>201</v>
       </c>
@@ -3785,7 +3791,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="39" spans="1:10" ht="28.9">
+    <row r="39" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
         <v>205</v>
       </c>
@@ -3808,7 +3814,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="40" spans="1:10" ht="28.9">
+    <row r="40" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
         <v>209</v>
       </c>
@@ -3831,7 +3837,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="41" spans="1:10" ht="28.9">
+    <row r="41" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
         <v>213</v>
       </c>
@@ -3854,7 +3860,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="42" spans="1:10" ht="43.15">
+    <row r="42" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
         <v>217</v>
       </c>
@@ -3881,8 +3887,10 @@
         <v>64</v>
       </c>
     </row>
-    <row r="43" spans="1:10" ht="15" customHeight="1">
-      <c r="A43" s="11"/>
+    <row r="43" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="11" t="s">
+        <v>371</v>
+      </c>
       <c r="B43" s="11" t="s">
         <v>83</v>
       </c>
@@ -3911,8 +3919,10 @@
         <v>90</v>
       </c>
     </row>
-    <row r="44" spans="1:10" ht="15" customHeight="1">
-      <c r="A44"/>
+    <row r="44" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="6" t="s">
+        <v>372</v>
+      </c>
       <c r="B44" s="11" t="s">
         <v>83</v>
       </c>
@@ -3941,7 +3951,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="45" spans="1:10" ht="28.9">
+    <row r="45" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A45" s="6">
         <v>5</v>
       </c>
@@ -3968,7 +3978,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="46" spans="1:10" s="8" customFormat="1" ht="14.45">
+    <row r="46" spans="1:10" s="8" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A46" s="7" t="s">
         <v>231</v>
       </c>
@@ -3993,7 +4003,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="47" spans="1:10" s="8" customFormat="1" ht="14.45">
+    <row r="47" spans="1:10" s="8" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
         <v>235</v>
       </c>
@@ -4018,7 +4028,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="48" spans="1:10" ht="28.9">
+    <row r="48" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A48" s="6">
         <v>6</v>
       </c>
@@ -4045,7 +4055,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="49" spans="1:10" ht="14.45">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" s="4">
         <v>7</v>
       </c>
@@ -4053,7 +4063,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="50" spans="1:10" ht="14.45">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
         <v>246</v>
       </c>
@@ -4076,7 +4086,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="51" spans="1:10" ht="14.45">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" s="4" t="s">
         <v>251</v>
       </c>
@@ -4102,7 +4112,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="52" spans="1:10" ht="14.45">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" s="4">
         <v>8</v>
       </c>
@@ -4128,7 +4138,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="53" spans="1:10" ht="57.6">
+    <row r="53" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A53" s="6">
         <v>9</v>
       </c>
@@ -4155,7 +4165,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="54" spans="1:10" ht="72">
+    <row r="54" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
         <v>267</v>
       </c>
@@ -4185,7 +4195,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="55" spans="1:10" ht="15" customHeight="1">
+    <row r="55" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>273</v>
       </c>
@@ -4217,7 +4227,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="56" spans="1:10" ht="15" customHeight="1">
+    <row r="56" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>277</v>
       </c>
@@ -4247,7 +4257,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="57" spans="1:10" ht="28.9">
+    <row r="57" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A57" s="4">
         <v>10</v>
       </c>
@@ -4273,7 +4283,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="58" spans="1:10" ht="15" customHeight="1">
+    <row r="58" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="11" t="s">
         <v>286</v>
       </c>
@@ -4301,7 +4311,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="59" spans="1:10" ht="15" customHeight="1">
+    <row r="59" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>290</v>
       </c>
@@ -4329,7 +4339,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="60" spans="1:10" ht="15" customHeight="1">
+    <row r="60" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>293</v>
       </c>
@@ -4357,7 +4367,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="61" spans="1:10" ht="28.9">
+    <row r="61" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A61" s="4">
         <v>11</v>
       </c>
@@ -4383,7 +4393,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="62" spans="1:10" ht="28.9">
+    <row r="62" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A62" s="4">
         <v>12</v>
       </c>
@@ -4409,7 +4419,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="63" spans="1:10" ht="14.45">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" s="4">
         <v>13</v>
       </c>
@@ -4435,7 +4445,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="64" spans="1:10" ht="57.6">
+    <row r="64" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="A64" s="4">
         <v>14</v>
       </c>
@@ -4461,7 +4471,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="65" spans="1:10" ht="28.9">
+    <row r="65" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A65" s="4">
         <v>15</v>
       </c>
@@ -4487,7 +4497,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="66" spans="1:10" ht="14.45">
+    <row r="66" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A66" s="4">
         <v>16</v>
       </c>
@@ -4513,7 +4523,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="67" spans="1:10" ht="57.6">
+    <row r="67" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A67" s="4">
         <v>17</v>
       </c>
@@ -4539,7 +4549,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="68" spans="1:10" ht="28.9">
+    <row r="68" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A68" s="4">
         <v>18</v>
       </c>
@@ -4565,7 +4575,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="69" spans="1:10" ht="14.45">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A69" s="4">
         <v>19</v>
       </c>
@@ -4588,7 +4598,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="70" spans="1:10" ht="37.5" customHeight="1">
+    <row r="70" spans="1:10" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>343</v>
       </c>
@@ -4618,31 +4628,31 @@
         <v>348</v>
       </c>
     </row>
-    <row r="71" spans="1:10" ht="15" customHeight="1">
+    <row r="71" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="11"/>
       <c r="B71" s="11"/>
       <c r="C71" s="11"/>
       <c r="D71" s="11"/>
     </row>
-    <row r="72" spans="1:10" ht="15" customHeight="1">
+    <row r="72" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72"/>
       <c r="B72" s="11"/>
       <c r="C72" s="11"/>
       <c r="D72" s="11"/>
     </row>
-    <row r="73" spans="1:10" ht="15" customHeight="1">
+    <row r="73" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73"/>
       <c r="B73" s="11"/>
       <c r="C73" s="11"/>
       <c r="D73" s="11"/>
     </row>
-    <row r="74" spans="1:10" ht="15" customHeight="1">
+    <row r="74" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74"/>
       <c r="B74" s="11"/>
       <c r="C74" s="11"/>
       <c r="D74" s="11"/>
     </row>
-    <row r="75" spans="1:10" ht="15" customHeight="1">
+    <row r="75" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75"/>
     </row>
   </sheetData>
@@ -4656,7 +4666,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{273AFAA3-99F7-4E93-9580-DCAE2B14D938}">
   <dimension ref="A1:G7"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.28515625" customWidth="1"/>
     <col min="2" max="2" width="18.42578125" customWidth="1"/>
@@ -4667,7 +4677,7 @@
     <col min="7" max="7" width="41.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="195.75" customHeight="1">
+    <row r="1" spans="1:7" ht="195.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>349</v>
       </c>
@@ -4690,7 +4700,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>351</v>
       </c>
@@ -4713,7 +4723,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="57.6">
+    <row r="3" spans="1:7" ht="75" x14ac:dyDescent="0.25">
       <c r="C3" t="s">
         <v>304</v>
       </c>
@@ -4730,7 +4740,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
         <v>359</v>
       </c>
@@ -4747,7 +4757,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
         <v>362</v>
       </c>
@@ -4764,7 +4774,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="43.15">
+    <row r="6" spans="1:7" ht="60" x14ac:dyDescent="0.25">
       <c r="C6" s="11" t="s">
         <v>364</v>
       </c>
@@ -4781,7 +4791,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
         <v>365</v>
       </c>
@@ -4808,20 +4818,20 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2489EBC-5098-4697-9724-F190D24E1C3D}">
   <dimension ref="A1:A5"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" ht="111" customHeight="1"/>
-    <row r="3" spans="1:1">
+    <row r="1" spans="1:1" ht="111" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>368</v>
       </c>
     </row>
-    <row r="4" spans="1:1">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>369</v>
       </c>
     </row>
-    <row r="5" spans="1:1">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>370</v>
       </c>
@@ -4833,15 +4843,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D5656983173B1142A9B62A9C329F89A7" ma:contentTypeVersion="13" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="71caa5f225d89a4181f0614974a0635b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="bb18a1b9-ddba-4244-9634-64732d0cb267" xmlns:ns3="06294a2e-6f87-4144-83b8-94a4d04d144a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d74eef483bec37fcdf125766e7bdb283" ns2:_="" ns3:_="">
     <xsd:import namespace="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
@@ -5048,6 +5049,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -5060,13 +5070,39 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148267B0-4CF5-48A7-B543-CDE45AF0A8FC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{226BE694-A00C-4E31-A532-690E39C51D9D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
+    <ds:schemaRef ds:uri="06294a2e-6f87-4144-83b8-94a4d04d144a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{226BE694-A00C-4E31-A532-690E39C51D9D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148267B0-4CF5-48A7-B543-CDE45AF0A8FC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E3A9028-3436-4B29-A420-9ED5B8A085B1}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E3A9028-3436-4B29-A420-9ED5B8A085B1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
+    <ds:schemaRef ds:uri="06294a2e-6f87-4144-83b8-94a4d04d144a"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Correction of concept tab to the logical model gets picked up
</commit_message>
<xml_diff>
--- a/input/requirements/Procedure.xlsx
+++ b/input/requirements/Procedure.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\edelman_nict1\IGs\GBB-IG\input\requirements\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahenket/Development/GitHub/Nictiz/GBB-IG/input/requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41642281-4408-4428-AC78-DE7A4991C766}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD2BF520-300F-7849-93DE-28B406CAEEF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="2" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
+    <workbookView xWindow="4880" yWindow="-35240" windowWidth="44340" windowHeight="30740" activeTab="1" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
   </bookViews>
   <sheets>
     <sheet name="Uitleg" sheetId="5" r:id="rId1"/>
@@ -42,195 +42,41 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
-    <author>Gijs de Haan</author>
     <author>tc={3FDD208F-8502-664C-BFA0-E27551C0A04E}</author>
     <author>tc={79B91D5E-D6C0-EB4C-A822-34BDEEC910A8}</author>
     <author>tc={B31F989E-38F1-9B49-B02D-1CA100C251B6}</author>
     <author>tc={02AB9C8B-2472-3B49-AFF6-EAEBBADFD826}</author>
   </authors>
   <commentList>
-    <comment ref="B5" authorId="0" shapeId="0" xr:uid="{0CE43E3D-F8D0-4D76-ADBB-DEDDAE3128A4}">
+    <comment ref="B6" authorId="0" shapeId="0" xr:uid="{3FDD208F-8502-664C-BFA0-E27551C0A04E}">
       <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Gijs de Haan:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Dienen de voorbeelden te gaan over informatiestandaarden waar het concept feitelijk wordt toegepast, of waar het toegepast zou kunnen worden.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B6" authorId="0" shapeId="0" xr:uid="{00E5C6E0-F5FB-4631-88A9-351F81EA32EF}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Gijs de Haan:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Wat wordt hier precies bedoeld?</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C6" authorId="1" shapeId="0" xr:uid="{3FDD208F-8502-664C-BFA0-E27551C0A04E}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[Opmerkingenthread]
+U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
+Opmerking:
     Dit met @Pieter Edelman bespreken. Van het basismodel worden gedurende de levensloop nieuwe instantiaties gemaakt, ik weet zelf niet zo goed wat dit voor effect heeft op de mapping van de informatiebehoefte.</t>
       </text>
     </comment>
-    <comment ref="B7" authorId="0" shapeId="0" xr:uid="{31D11400-82E7-40E5-9619-2E80D24042E8}">
+    <comment ref="B7" authorId="1" shapeId="0" xr:uid="{79B91D5E-D6C0-EB4C-A822-34BDEEC910A8}">
       <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Gijs de Haan:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Gaat het om alle bij de teamleden bekende synoniemen, of om 'alle' in absolute zin. 
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Dienen het sematische equivalente synoniemen te zijn, of synoniemen in de meer algemene betekenis?
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Jacob: vallen specialisaties hier ook onder (zoals verplaagkundige intervanties)</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C7" authorId="2" shapeId="0" xr:uid="{79B91D5E-D6C0-EB4C-A822-34BDEEC910A8}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[Opmerkingenthread]
+U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
+Opmerking:
     (Verpleegkundige) Interventie</t>
       </text>
     </comment>
-    <comment ref="B9" authorId="0" shapeId="0" xr:uid="{22F42EEB-7750-45F3-8F49-8E202FD8AEA5}">
+    <comment ref="B9" authorId="2" shapeId="0" xr:uid="{B31F989E-38F1-9B49-B02D-1CA100C251B6}">
       <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Gijs de Haan:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Is het de bedoeling om een volledige opsomming van onjuist gebruik te geven, of alleen (typische) voorbeelden van onjuist gebruik.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C9" authorId="3" shapeId="0" xr:uid="{B31F989E-38F1-9B49-B02D-1CA100C251B6}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[Opmerkingenthread]
+U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
+Opmerking:
     Ik denk: verpleegkundige interventies juist wel. Misschien tussen haakjes toekomst?</t>
       </text>
     </comment>
-    <comment ref="C10" authorId="4" shapeId="0" xr:uid="{02AB9C8B-2472-3B49-AFF6-EAEBBADFD826}">
+    <comment ref="B10" authorId="3" shapeId="0" xr:uid="{02AB9C8B-2472-3B49-AFF6-EAEBBADFD826}">
       <text>
-        <t xml:space="preserve">[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t xml:space="preserve">[Opmerkingenthread]
+U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
+Opmerking:
     EEHRXf logical model EHDSProcedure </t>
       </text>
     </comment>
@@ -256,94 +102,94 @@
   <commentList>
     <comment ref="I2" authorId="0" shapeId="0" xr:uid="{5A89DE7A-12B0-4853-A72C-C1F8CE807912}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[Opmerkingenthread]
+U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
+Opmerking:
     Antwoord Jacob: Het is alleen van toepassing als het onderwerp (in dit geval de verrichting dus) een tijdsverloop heeft. Dus het moet een gebeurtenis of een handeling zijn. Zoals: verrichting, afspraak, ontmoeting, aandoening. Bij deze onderwerpen speelt de vraag: moet het gezochte model (of de gezochte modellen) geschikt zijn voor handelingen/gebeurtenissen in het verleden, nog lopende handelingen/gebeurtenissen, en/of toekomstige?
-Reply:
+Beantwoorden:
     is het requirement van toepassing op verrichtingen in het verleden, lopende verrichtingen, en/of toekomstige verrichtingen</t>
       </text>
     </comment>
     <comment ref="C10" authorId="1" shapeId="0" xr:uid="{6AE4750B-1627-475B-AD11-9F1CF1D6EB01}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[Opmerkingenthread]
+U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
+Opmerking:
     Hoort in bouwblok Service Request denk ik?</t>
       </text>
     </comment>
     <comment ref="D11" authorId="2" shapeId="0" xr:uid="{7ED1F6D6-CBC1-4F3F-91C6-B1EE1DC523F6}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[Opmerkingenthread]
+U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
+Opmerking:
     Niet zeker hoe Procedure.performed anders is dan time</t>
       </text>
     </comment>
     <comment ref="E12" authorId="3" shapeId="0" xr:uid="{4821E63C-4957-4B36-8174-ADC6AD9685DA}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[Opmerkingenthread]
+U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
+Opmerking:
     Deze informatiebehoefte lijkt buiten de scope van dit bouwblok te vallen</t>
       </text>
     </comment>
     <comment ref="G21" authorId="4" shapeId="0" xr:uid="{5C8C418A-E02E-4604-BC23-98C9785EB5EF}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[Opmerkingenthread]
+U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
+Opmerking:
     Ik mis hier de SNOMED binding (preferred) uit het EHDS model.</t>
       </text>
     </comment>
     <comment ref="C45" authorId="5" shapeId="0" xr:uid="{59F7D42D-131B-4727-A027-46A3E6A6ADC1}">
       <text>
-        <t xml:space="preserve">[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t xml:space="preserve">[Opmerkingenthread]
+U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
+Opmerking:
     Blijft dit bestaan als de procedure is afgerond?
-Reply:
+Beantwoorden:
     Ik zie dat in de pilot Afsprakenmodel.pdf er een mapping is gemaakt naar “Reference model - Facility” en dan een verwijzing naar Location (FHIR). Ik ga (Wouter) vragen hoe dit zit.
 </t>
       </text>
     </comment>
     <comment ref="A46" authorId="6" shapeId="0" xr:uid="{9F26CE90-3C21-415F-9801-18060348C83A}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[Opmerkingenthread]
+U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
+Opmerking:
     Verwijzing naar bouwblok Locatie waar deze twee gegevens vastgelegd worden</t>
       </text>
     </comment>
     <comment ref="G57" authorId="7" shapeId="0" xr:uid="{25CD8BD5-27EA-4E72-9F13-5AD9AE8ECD9F}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[Opmerkingenthread]
+U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
+Opmerking:
     Dit is de variabiliteit volgens het FHIR resource; we hoeven echter niet méér mee te nemen dan waar informatiebehoefte voor is (zie commentaar bij spelregel https://nictiz.atlassian.net/browse/DAGIM-19?focusedCommentId=221118)</t>
       </text>
     </comment>
     <comment ref="E62" authorId="8" shapeId="0" xr:uid="{50562775-F32C-4F82-849B-F523FED9660E}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[Opmerkingenthread]
+U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
+Opmerking:
     Wij denken dat dit bij het bouwblok Encounter zou moeten</t>
       </text>
     </comment>
     <comment ref="G67" authorId="9" shapeId="0" xr:uid="{A7AE4957-8562-4CAB-811C-FA102CEC5345}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[Opmerkingenthread]
+U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
+Opmerking:
     nieuwe versie EHDSProcedure is dit een codeableConcept</t>
       </text>
     </comment>
     <comment ref="E68" authorId="10" shapeId="0" xr:uid="{18F12EB5-0AEE-44F9-A577-4C34B2D010C7}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[Opmerkingenthread]
+U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
+Opmerking:
     Was voorheen notitie/commentaar</t>
       </text>
     </comment>
@@ -359,9 +205,9 @@
   <commentList>
     <comment ref="C3" authorId="0" shapeId="0" xr:uid="{97F18402-58BF-4CEB-8CE0-124364433627}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[Opmerkingenthread]
+U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
+Opmerking:
     Wij denken dat dit bij het bouwblok Encounter zou moeten</t>
       </text>
     </comment>
@@ -370,7 +216,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="373">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="367">
   <si>
     <t>Veld</t>
   </si>
@@ -381,63 +227,42 @@
     <t>Conceptbeschrijving</t>
   </si>
   <si>
-    <t>[De definitie of beschrijving van het concept.]</t>
-  </si>
-  <si>
     <t>Het concept Verrichting beschrijft een therapeutische of diagnostische verrichting, die de patiënt heeft ondergaan of zal ondergaan.</t>
   </si>
   <si>
     <t>Doel</t>
   </si>
   <si>
-    <t>[De doelen en redenen om het concept vast te leggen en/of uit te wisselen.]</t>
-  </si>
-  <si>
     <t>Een verrichting wordt uitgevoerd of gepland in het kader van een uitgezet beleid of voor het verkrijgen van aanvullende informatie in het diagnostisch proces. Het vastleggen van verrichtingen dient om inzicht te krijgen in de behandeling van de patiënt. Daarnaast worden verrichtingen vastgelegd ten behoeve van administratieve doeleinden zoals facturering en werklastmeting, wetenschappelijk onderzoek en/of onderwijs.</t>
   </si>
   <si>
     <t>Gebruiksscenario(’s)</t>
   </si>
   <si>
-    <t>[Geeft aan in welke context(en) het concept wordt gebruikt. Geef voorbeelden van gebruik in informatiestandaarden.]</t>
-  </si>
-  <si>
     <t>Uitgevoerde en toekomstige therapeutische en diagnostische verrichtingen. Bijvoorbeeld in de informatiestandaarden Geboortezorg, Acute zorg, Huisartsenzorg, BgZ-MSZ en eOverdracht.</t>
   </si>
   <si>
     <t>Representatie</t>
   </si>
   <si>
-    <t>[Beschrijf hier wat er voor de dossiervorming belangrijk is rondom de levenscyclus en instantiaties van het concept.]</t>
-  </si>
-  <si>
     <t>Zie comment.</t>
   </si>
   <si>
     <t>Alias(sen)</t>
   </si>
   <si>
-    <t>[Alle bekende synoniemen voor het concept.]</t>
-  </si>
-  <si>
     <t>Behandeling (dekt maar een deel van het concept verrichting)</t>
   </si>
   <si>
     <t>Juist gebruik</t>
   </si>
   <si>
-    <t>[Beschrijf hier waarvoor het concept wél bedoeld is].</t>
-  </si>
-  <si>
     <t>Het concept is bedoeld voor het vastleggen van therapeutische en diagnostische verrichtingen.</t>
   </si>
   <si>
     <t>Onjuist gebruik</t>
   </si>
   <si>
-    <t>[Beschrijf hier waar het concept niet voor bedoeld is, en geef waar mogelijk aan welk concept er wel geschikt voor is.]</t>
-  </si>
-  <si>
     <t>Het concept is niet bedoeld voor het vastleggen van verpleegkundige verrichtingen, administratieve verrichtingen en dat wat niet een verrichting is. Hiervoor zijn nog geen generieke bouwblokken ontwikkeld.</t>
   </si>
   <si>
@@ -445,9 +270,6 @@
   </si>
   <si>
     <t>Referenties</t>
-  </si>
-  <si>
-    <t>[Relevante bronstandaarden of informatiebronnen die het ontwerp en de scope van het concept hebben beïnvloed.]</t>
   </si>
   <si>
     <t>Zibs, Geboortezorg, JGZ, Acute zorg, Huisartsenzorg, BgZ-MSZ, eOverdracht</t>
@@ -1493,13 +1315,19 @@
   </si>
   <si>
     <t>4.2.2</t>
+  </si>
+  <si>
+    <t>ART-DECOR-id</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.4.3.11.60.153.4.28/2026-07-15T00:00:00</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1531,37 +1359,11 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="9"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color rgb="FF000000"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF000000"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -1590,7 +1392,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1632,15 +1434,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2360,7 +2159,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Kantoorthema">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -2676,19 +2475,19 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="C6" dT="2026-06-11T12:39:40.67" personId="{B78312EE-1EC2-432E-85A4-5F27F7CE82CD}" id="{3FDD208F-8502-664C-BFA0-E27551C0A04E}">
+  <threadedComment ref="B6" dT="2026-06-11T12:39:40.67" personId="{B78312EE-1EC2-432E-85A4-5F27F7CE82CD}" id="{3FDD208F-8502-664C-BFA0-E27551C0A04E}">
     <text>Dit met @Pieter Edelman bespreken. Van het basismodel worden gedurende de levensloop nieuwe instantiaties gemaakt, ik weet zelf niet zo goed wat dit voor effect heeft op de mapping van de informatiebehoefte.</text>
     <mentions>
       <mention mentionpersonId="{813D4FC9-CFB5-F94C-ADA7-DB3F2E9D5D63}" mentionId="{6B8FA3A7-D49F-654F-AD4B-6AAD557E2ABA}" startIndex="8" length="15"/>
     </mentions>
   </threadedComment>
-  <threadedComment ref="C7" dT="2026-06-11T12:24:44.12" personId="{B78312EE-1EC2-432E-85A4-5F27F7CE82CD}" id="{79B91D5E-D6C0-EB4C-A822-34BDEEC910A8}">
+  <threadedComment ref="B7" dT="2026-06-11T12:24:44.12" personId="{B78312EE-1EC2-432E-85A4-5F27F7CE82CD}" id="{79B91D5E-D6C0-EB4C-A822-34BDEEC910A8}">
     <text>(Verpleegkundige) Interventie</text>
   </threadedComment>
-  <threadedComment ref="C9" dT="2026-06-11T12:30:38.96" personId="{B78312EE-1EC2-432E-85A4-5F27F7CE82CD}" id="{B31F989E-38F1-9B49-B02D-1CA100C251B6}">
+  <threadedComment ref="B9" dT="2026-06-11T12:30:38.96" personId="{B78312EE-1EC2-432E-85A4-5F27F7CE82CD}" id="{B31F989E-38F1-9B49-B02D-1CA100C251B6}">
     <text>Ik denk: verpleegkundige interventies juist wel. Misschien tussen haakjes toekomst?</text>
   </threadedComment>
-  <threadedComment ref="C10" dT="2026-06-11T12:34:15.65" personId="{B78312EE-1EC2-432E-85A4-5F27F7CE82CD}" id="{02AB9C8B-2472-3B49-AFF6-EAEBBADFD826}">
+  <threadedComment ref="B10" dT="2026-06-11T12:34:15.65" personId="{B78312EE-1EC2-432E-85A4-5F27F7CE82CD}" id="{02AB9C8B-2472-3B49-AFF6-EAEBBADFD826}">
     <text xml:space="preserve">EEHRXf logical model EHDSProcedure </text>
   </threadedComment>
 </ThreadedComments>
@@ -2756,12 +2555,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F1013F7-63B2-4F83-92B0-1C8153859891}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="218.42578125" customWidth="1"/>
+    <col min="1" max="1" width="218.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3"/>
     </row>
   </sheetData>
@@ -2772,19 +2571,19 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CC1E3B3-D087-4A2B-920B-9BA971FAD64B}">
-  <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="191" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="2" width="32.7109375" customWidth="1"/>
-    <col min="3" max="3" width="58.42578125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="99.85546875" style="3" customWidth="1"/>
+    <col min="2" max="2" width="59.6640625" customWidth="1"/>
+    <col min="3" max="3" width="58.5" style="3" customWidth="1"/>
+    <col min="4" max="4" width="99.83203125" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="190.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="191" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3"/>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="15" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -2792,98 +2591,82 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="32" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="18" t="s">
+    </row>
+    <row r="4" spans="1:3" ht="96" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="105" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="B4" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="17" t="s">
+    </row>
+    <row r="5" spans="1:3" ht="48" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="B5" s="17" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="6" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B6" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="18" t="s">
+    </row>
+    <row r="7" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="B7" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="17" t="s">
+    </row>
+    <row r="8" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="B8" s="17" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="9" spans="1:3" ht="80" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="17" t="s">
+      <c r="B9" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C9" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="10" spans="1:3" ht="64" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="17" t="s">
+      <c r="B10" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C10" s="3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" s="18" t="s">
-        <v>22</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>24</v>
-      </c>
-      <c r="B10" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="C10" s="18" t="s">
-        <v>26</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>27</v>
+    <row r="11" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>365</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>366</v>
       </c>
     </row>
   </sheetData>
@@ -2896,54 +2679,54 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7034CDAF-2A08-4BE8-92C3-F4E7A6F24E1B}">
   <dimension ref="A1:K75"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="22.42578125" style="4" customWidth="1"/>
-    <col min="3" max="3" width="14.85546875" style="4" customWidth="1"/>
+    <col min="1" max="2" width="22.5" style="4" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" style="4" customWidth="1"/>
     <col min="4" max="4" width="17" style="4" customWidth="1"/>
     <col min="5" max="5" width="38" customWidth="1"/>
-    <col min="6" max="6" width="68.42578125" customWidth="1"/>
-    <col min="7" max="7" width="52.140625" customWidth="1"/>
-    <col min="8" max="9" width="48.7109375" customWidth="1"/>
-    <col min="10" max="10" width="34.42578125" customWidth="1"/>
-    <col min="11" max="11" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="68.5" customWidth="1"/>
+    <col min="7" max="7" width="52.1640625" customWidth="1"/>
+    <col min="8" max="9" width="48.6640625" customWidth="1"/>
+    <col min="10" max="10" width="34.5" customWidth="1"/>
+    <col min="11" max="11" width="19.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="88.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="88.5" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="J2" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C2" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="D2" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>37</v>
-      </c>
       <c r="K2" s="2"/>
     </row>
-    <row r="3" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A3" s="6">
         <v>1</v>
       </c>
@@ -2951,431 +2734,431 @@
       <c r="C3" s="6"/>
       <c r="D3" s="6"/>
       <c r="E3" s="3" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="B4" s="6"/>
       <c r="C4" s="6" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="F4" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G4" t="s">
         <v>39</v>
       </c>
-      <c r="G4" t="s">
-        <v>47</v>
-      </c>
       <c r="H4" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="G5" t="s">
+        <v>39</v>
+      </c>
+      <c r="H5" t="s">
+        <v>39</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="32" x14ac:dyDescent="0.2">
+      <c r="A6" s="6" t="s">
         <v>44</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="G5" t="s">
-        <v>47</v>
-      </c>
-      <c r="H5" t="s">
-        <v>47</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="45" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
-        <v>52</v>
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="6" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="48" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="B8" s="6"/>
       <c r="C8" s="6" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="J8" s="3"/>
     </row>
-    <row r="9" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="6" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="D9" s="6"/>
       <c r="E9" s="3" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
       <c r="D10" s="6"/>
       <c r="E10" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>74</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="E11" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="F11" s="13" t="s">
         <v>78</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="G11" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="G10" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="H10" s="3" t="s">
+      <c r="H11" t="s">
         <v>80</v>
       </c>
-      <c r="J10" s="3" t="s">
+      <c r="I11" s="11" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="J11" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="B11" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="C11" s="11" t="s">
-        <v>84</v>
-      </c>
-      <c r="D11" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="E11" s="13" t="s">
-        <v>85</v>
-      </c>
-      <c r="F11" s="13" t="s">
-        <v>86</v>
-      </c>
-      <c r="G11" s="13" t="s">
-        <v>87</v>
-      </c>
-      <c r="H11" t="s">
-        <v>88</v>
-      </c>
-      <c r="I11" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="J11" s="12" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A12" s="4">
         <v>2</v>
       </c>
       <c r="E12" t="s">
+        <v>83</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="J12" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A13" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="E13" t="s">
+        <v>89</v>
+      </c>
+      <c r="F13" t="s">
+        <v>90</v>
+      </c>
+      <c r="G13" t="s">
+        <v>39</v>
+      </c>
+      <c r="H13" t="s">
         <v>91</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="J13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A14" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="G12" s="3" t="s">
+      <c r="E14" t="s">
         <v>93</v>
       </c>
-      <c r="H12" s="3" t="s">
+      <c r="F14" t="s">
         <v>94</v>
       </c>
-      <c r="J12" t="s">
+      <c r="G14" t="s">
+        <v>39</v>
+      </c>
+      <c r="H14" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
+      <c r="J14" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A15" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E15" t="s">
         <v>97</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F15" t="s">
         <v>98</v>
       </c>
-      <c r="G13" t="s">
-        <v>47</v>
-      </c>
-      <c r="H13" t="s">
+      <c r="G15" t="s">
+        <v>39</v>
+      </c>
+      <c r="H15" t="s">
         <v>99</v>
       </c>
-      <c r="J13" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="E14" t="s">
-        <v>101</v>
-      </c>
-      <c r="F14" t="s">
-        <v>102</v>
-      </c>
-      <c r="G14" t="s">
-        <v>47</v>
-      </c>
-      <c r="H14" t="s">
-        <v>103</v>
-      </c>
-      <c r="J14" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="E15" t="s">
-        <v>105</v>
-      </c>
-      <c r="F15" t="s">
-        <v>106</v>
-      </c>
-      <c r="G15" t="s">
-        <v>47</v>
-      </c>
-      <c r="H15" t="s">
-        <v>107</v>
-      </c>
       <c r="J15" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" s="4">
         <v>3</v>
       </c>
       <c r="E16" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="F16" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="J16" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="B17" s="6"/>
       <c r="C17" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="E17" t="s">
+        <v>104</v>
+      </c>
+      <c r="F17" t="s">
+        <v>105</v>
+      </c>
+      <c r="G17" t="s">
+        <v>106</v>
+      </c>
+      <c r="H17" t="s">
+        <v>107</v>
+      </c>
+      <c r="J17" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A18" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="E18" t="s">
+        <v>110</v>
+      </c>
+      <c r="F18" t="s">
         <v>111</v>
       </c>
-      <c r="D17" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="E17" t="s">
+      <c r="G18" t="s">
         <v>112</v>
       </c>
-      <c r="F17" t="s">
+      <c r="H18" t="s">
         <v>113</v>
       </c>
-      <c r="G17" t="s">
+      <c r="J18" t="s">
         <v>114</v>
       </c>
-      <c r="H17" t="s">
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A19" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="J17" t="s">
+      <c r="C19" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="E19" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="s">
+      <c r="F19" t="s">
         <v>117</v>
       </c>
-      <c r="D18" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="E18" t="s">
+      <c r="G19" t="s">
         <v>118</v>
       </c>
-      <c r="F18" t="s">
+      <c r="H19" t="s">
         <v>119</v>
       </c>
-      <c r="G18" t="s">
+      <c r="J19" t="s">
         <v>120</v>
       </c>
-      <c r="H18" t="s">
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A20" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="J18" t="s">
+      <c r="C20" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="E20" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A19" s="4" t="s">
+      <c r="F20" t="s">
         <v>123</v>
       </c>
-      <c r="C19" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="E19" t="s">
+      <c r="G20" t="s">
         <v>124</v>
       </c>
-      <c r="F19" t="s">
-        <v>125</v>
-      </c>
-      <c r="G19" t="s">
-        <v>126</v>
-      </c>
-      <c r="H19" t="s">
-        <v>127</v>
-      </c>
-      <c r="J19" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A20" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="E20" t="s">
-        <v>130</v>
-      </c>
-      <c r="F20" t="s">
-        <v>131</v>
-      </c>
-      <c r="G20" t="s">
-        <v>132</v>
-      </c>
       <c r="H20" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="J20" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="48" x14ac:dyDescent="0.2">
       <c r="A21" s="6">
         <v>4</v>
       </c>
@@ -3383,1276 +3166,1276 @@
       <c r="C21" s="6"/>
       <c r="D21" s="6"/>
       <c r="E21" s="3" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" s="6" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="B22" s="6"/>
       <c r="C22" s="6" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="F22" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="H22" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="G22" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="H22" s="3" t="s">
-        <v>142</v>
-      </c>
       <c r="J22" s="3"/>
     </row>
-    <row r="23" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A23" s="6" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="B23" s="6"/>
       <c r="C23" s="6"/>
       <c r="D23" s="6"/>
       <c r="E23" s="3" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A24" s="6" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="B24" s="6"/>
       <c r="C24" s="6"/>
       <c r="D24" s="6"/>
       <c r="E24" s="3" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="G24" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="H24" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="J24" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+      <c r="A25" s="6" t="s">
         <v>141</v>
-      </c>
-      <c r="H24" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="J24" s="3" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A25" s="6" t="s">
-        <v>149</v>
       </c>
       <c r="B25" s="6"/>
       <c r="C25" s="6"/>
       <c r="D25" s="6"/>
       <c r="E25" s="3" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A26" s="6" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="6"/>
       <c r="D26" s="6"/>
       <c r="E26" s="3" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="F26" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A27" s="6" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="B27" s="6"/>
       <c r="C27" s="6"/>
       <c r="D27" s="6"/>
       <c r="E27" s="3" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="F27" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A28" s="6" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="B28" s="6"/>
       <c r="C28" s="6"/>
       <c r="D28" s="6"/>
       <c r="E28" s="3" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="F28" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A29" s="6" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="B29" s="6"/>
       <c r="C29" s="6"/>
       <c r="D29" s="6"/>
       <c r="E29" s="3" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="F29" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A30" s="6" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="B30" s="6"/>
       <c r="C30" s="6"/>
       <c r="D30" s="6"/>
       <c r="E30" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="F30" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A31" s="6" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="B31" s="6"/>
       <c r="C31" s="6"/>
       <c r="D31" s="6"/>
       <c r="E31" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="F31" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="J31" s="3" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A32" s="6" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="B32" s="6"/>
       <c r="C32" s="6"/>
       <c r="D32" s="6"/>
       <c r="E32" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="F32" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="J32" s="3" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A33" s="6" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="B33" s="6"/>
       <c r="C33" s="6"/>
       <c r="D33" s="6"/>
       <c r="E33" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="F33" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A34" s="6" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="B34" s="6"/>
       <c r="C34" s="6"/>
       <c r="D34" s="6"/>
       <c r="E34" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="F34" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="H34" s="3" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="J34" s="3" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A35" s="6" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="B35" s="6"/>
       <c r="C35" s="6"/>
       <c r="D35" s="6"/>
       <c r="E35" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="F35" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="H35" s="3" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="J35" s="3" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A36" s="6" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="B36" s="6"/>
       <c r="C36" s="6"/>
       <c r="D36" s="6"/>
       <c r="E36" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="F36" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="H36" s="3" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="J36" s="3" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A37" s="6" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="6"/>
       <c r="D37" s="6"/>
       <c r="E37" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="F37" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="H37" s="3" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="J37" s="3" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A38" s="6" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="B38" s="6"/>
       <c r="C38" s="6"/>
       <c r="D38" s="6"/>
       <c r="E38" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="F38" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="G38" s="3" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="H38" s="3" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="J38" s="3" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A39" s="6" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="B39" s="6"/>
       <c r="C39" s="6"/>
       <c r="D39" s="6"/>
       <c r="E39" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="F39" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="J39" s="3" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A40" s="6" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="B40" s="6"/>
       <c r="C40" s="6"/>
       <c r="D40" s="6"/>
       <c r="E40" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="F40" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="G40" s="3" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="H40" s="3" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="J40" s="3" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A41" s="6" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="B41" s="6"/>
       <c r="C41" s="6"/>
       <c r="D41" s="6"/>
       <c r="E41" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="F41" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="H41" s="3" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="J41" s="3" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" ht="48" x14ac:dyDescent="0.2">
       <c r="A42" s="6" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="B42" s="6"/>
       <c r="C42" s="6" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="F42" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="G42" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H42" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="G42" s="3" t="s">
-        <v>219</v>
-      </c>
-      <c r="H42" s="3" t="s">
-        <v>142</v>
-      </c>
       <c r="J42" s="3" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="11" t="s">
-        <v>371</v>
+        <v>363</v>
       </c>
       <c r="B43" s="11" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="C43" s="11" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="E43" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="F43" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="G43" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="H43" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="I43" s="11" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="J43" s="12" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="6" t="s">
-        <v>372</v>
+        <v>364</v>
       </c>
       <c r="B44" s="11" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="C44" s="11" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="D44" s="11" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="E44" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
       <c r="F44" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="G44" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="H44" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="I44" s="11" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="J44" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A45" s="6">
         <v>5</v>
       </c>
       <c r="B45" s="6"/>
       <c r="C45" s="6" t="s">
-        <v>226</v>
+        <v>218</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
       <c r="H45" s="3" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="J45" s="3" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" s="8" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A46" s="7" t="s">
-        <v>231</v>
+        <v>223</v>
       </c>
       <c r="B46" s="7"/>
       <c r="C46" s="7"/>
       <c r="D46" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="E46" t="s">
+        <v>224</v>
+      </c>
+      <c r="F46" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="G46" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="H46" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="J46" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A47" s="7" t="s">
         <v>227</v>
-      </c>
-      <c r="E46" t="s">
-        <v>232</v>
-      </c>
-      <c r="F46" s="8" t="s">
-        <v>233</v>
-      </c>
-      <c r="G46" s="8" t="s">
-        <v>234</v>
-      </c>
-      <c r="H46" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="J46" s="9" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" s="8" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A47" s="7" t="s">
-        <v>235</v>
       </c>
       <c r="B47" s="7"/>
       <c r="C47" s="7"/>
       <c r="D47" s="6" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
       <c r="E47" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="F47" s="8" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="H47" s="8" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="J47" s="8" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A48" s="6">
         <v>6</v>
       </c>
       <c r="B48" s="6"/>
       <c r="C48" s="6" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>243</v>
+        <v>235</v>
       </c>
       <c r="G48" s="3" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
       <c r="H48" s="3" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="J48" s="3" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A49" s="4">
         <v>7</v>
       </c>
       <c r="E49" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A50" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="E50" t="s">
+        <v>240</v>
+      </c>
+      <c r="F50" t="s">
+        <v>241</v>
+      </c>
+      <c r="G50" t="s">
+        <v>242</v>
+      </c>
+      <c r="H50" t="s">
+        <v>128</v>
+      </c>
+      <c r="J50" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A51" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="D51" s="4" t="s">
         <v>245</v>
       </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A50" s="4" t="s">
+      <c r="E51" t="s">
         <v>246</v>
       </c>
-      <c r="C50" s="4" t="s">
+      <c r="F51" t="s">
         <v>247</v>
       </c>
-      <c r="E50" t="s">
+      <c r="G51" t="s">
         <v>248</v>
       </c>
-      <c r="F50" t="s">
-        <v>249</v>
-      </c>
-      <c r="G50" t="s">
-        <v>250</v>
-      </c>
-      <c r="H50" t="s">
-        <v>136</v>
-      </c>
-      <c r="J50" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A51" s="4" t="s">
-        <v>251</v>
-      </c>
-      <c r="C51" s="4" t="s">
-        <v>252</v>
-      </c>
-      <c r="D51" s="4" t="s">
-        <v>253</v>
-      </c>
-      <c r="E51" t="s">
-        <v>254</v>
-      </c>
-      <c r="F51" t="s">
-        <v>255</v>
-      </c>
-      <c r="G51" t="s">
-        <v>256</v>
-      </c>
       <c r="H51" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="J51" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A52" s="4">
         <v>8</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="E52" t="s">
-        <v>259</v>
+        <v>251</v>
       </c>
       <c r="F52" t="s">
-        <v>260</v>
+        <v>252</v>
       </c>
       <c r="G52" t="s">
-        <v>261</v>
+        <v>253</v>
       </c>
       <c r="H52" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="J52" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" ht="64" x14ac:dyDescent="0.2">
       <c r="A53" s="6">
         <v>9</v>
       </c>
       <c r="B53" s="6"/>
       <c r="C53" s="6" t="s">
-        <v>263</v>
+        <v>255</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="E53" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="F53" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="G53" s="3">
         <v>0</v>
       </c>
       <c r="H53" s="3" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="J53" s="3" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" ht="75" x14ac:dyDescent="0.25">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" ht="80" x14ac:dyDescent="0.2">
       <c r="A54" s="4" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
       <c r="B54" s="11" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="C54" s="11"/>
       <c r="D54" s="11" t="s">
+        <v>260</v>
+      </c>
+      <c r="E54" s="11" t="s">
+        <v>260</v>
+      </c>
+      <c r="F54" s="11" t="s">
+        <v>261</v>
+      </c>
+      <c r="G54" s="11" t="s">
+        <v>262</v>
+      </c>
+      <c r="H54" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="I54" s="11" t="s">
+        <v>263</v>
+      </c>
+      <c r="J54" s="12" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>265</v>
+      </c>
+      <c r="B55" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="C55" s="11" t="s">
+        <v>266</v>
+      </c>
+      <c r="D55" s="11" t="s">
+        <v>260</v>
+      </c>
+      <c r="E55" t="s">
+        <v>267</v>
+      </c>
+      <c r="F55" t="s">
         <v>268</v>
       </c>
-      <c r="E54" s="11" t="s">
-        <v>268</v>
-      </c>
-      <c r="F54" s="11" t="s">
+      <c r="G55" t="s">
+        <v>216</v>
+      </c>
+      <c r="H55" t="s">
+        <v>80</v>
+      </c>
+      <c r="I55" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="J55" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
         <v>269</v>
       </c>
-      <c r="G54" s="11" t="s">
+      <c r="B56" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="C56" s="11" t="s">
         <v>270</v>
-      </c>
-      <c r="H54" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="I54" s="11" t="s">
-        <v>271</v>
-      </c>
-      <c r="J54" s="12" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>273</v>
-      </c>
-      <c r="B55" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="C55" s="11" t="s">
-        <v>274</v>
-      </c>
-      <c r="D55" s="11" t="s">
-        <v>268</v>
-      </c>
-      <c r="E55" t="s">
-        <v>275</v>
-      </c>
-      <c r="F55" t="s">
-        <v>276</v>
-      </c>
-      <c r="G55" t="s">
-        <v>224</v>
-      </c>
-      <c r="H55" t="s">
-        <v>88</v>
-      </c>
-      <c r="I55" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="J55" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
-        <v>277</v>
-      </c>
-      <c r="B56" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="C56" s="11" t="s">
-        <v>278</v>
       </c>
       <c r="D56" s="11"/>
       <c r="E56" s="13" t="s">
-        <v>279</v>
+        <v>271</v>
       </c>
       <c r="F56" s="13" t="s">
-        <v>280</v>
+        <v>272</v>
       </c>
       <c r="G56" s="13" t="s">
-        <v>281</v>
+        <v>273</v>
       </c>
       <c r="H56" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="I56" s="11" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="J56" s="12" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A57" s="4">
         <v>10</v>
       </c>
       <c r="C57" t="s">
-        <v>282</v>
+        <v>274</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>283</v>
+        <v>275</v>
       </c>
       <c r="E57" t="s">
-        <v>282</v>
+        <v>274</v>
       </c>
       <c r="F57" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="G57" s="10" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="H57" s="3" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="J57" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="58" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="11" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="B58" s="11" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="C58" s="11"/>
       <c r="D58" s="11"/>
       <c r="E58" s="11" t="s">
-        <v>287</v>
+        <v>279</v>
       </c>
       <c r="F58" s="11" t="s">
-        <v>288</v>
+        <v>280</v>
       </c>
       <c r="G58" s="11" t="s">
-        <v>289</v>
+        <v>281</v>
       </c>
       <c r="H58" s="11" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="I58" s="11" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="J58" s="12" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>290</v>
+        <v>282</v>
       </c>
       <c r="B59" s="11" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="C59" s="11"/>
       <c r="D59" s="11"/>
       <c r="E59" s="13" t="s">
-        <v>282</v>
+        <v>274</v>
       </c>
       <c r="F59" s="13" t="s">
-        <v>291</v>
+        <v>283</v>
       </c>
       <c r="G59" s="13" t="s">
-        <v>292</v>
+        <v>284</v>
       </c>
       <c r="H59" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="I59" s="11" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="J59" s="12" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="60" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>293</v>
+        <v>285</v>
       </c>
       <c r="B60" s="11" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="C60" s="11"/>
       <c r="D60" s="11"/>
       <c r="E60" t="s">
-        <v>294</v>
+        <v>286</v>
       </c>
       <c r="F60" t="s">
-        <v>295</v>
+        <v>287</v>
       </c>
       <c r="G60" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="H60" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="I60" s="11" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="J60" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A61" s="4">
         <v>11</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>297</v>
+        <v>289</v>
       </c>
       <c r="D61" s="4" t="s">
-        <v>298</v>
+        <v>290</v>
       </c>
       <c r="E61" t="s">
-        <v>299</v>
+        <v>291</v>
       </c>
       <c r="F61" t="s">
-        <v>300</v>
+        <v>292</v>
       </c>
       <c r="G61" t="s">
-        <v>301</v>
+        <v>293</v>
       </c>
       <c r="H61" s="3" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="J61" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A62" s="4">
         <v>12</v>
       </c>
       <c r="C62" s="4" t="s">
+        <v>289</v>
+      </c>
+      <c r="D62" s="4" t="s">
+        <v>295</v>
+      </c>
+      <c r="E62" t="s">
+        <v>296</v>
+      </c>
+      <c r="F62" t="s">
         <v>297</v>
       </c>
-      <c r="D62" s="4" t="s">
-        <v>303</v>
-      </c>
-      <c r="E62" t="s">
-        <v>304</v>
-      </c>
-      <c r="F62" t="s">
-        <v>305</v>
-      </c>
       <c r="G62" t="s">
-        <v>306</v>
+        <v>298</v>
       </c>
       <c r="H62" s="3" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="J62" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A63" s="4">
         <v>13</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>307</v>
+        <v>299</v>
       </c>
       <c r="D63" s="4" t="s">
-        <v>297</v>
+        <v>289</v>
       </c>
       <c r="E63" t="s">
-        <v>308</v>
+        <v>300</v>
       </c>
       <c r="F63" t="s">
-        <v>309</v>
+        <v>301</v>
       </c>
       <c r="G63" t="s">
-        <v>310</v>
+        <v>302</v>
       </c>
       <c r="H63" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="J63" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10" ht="75" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" ht="64" x14ac:dyDescent="0.2">
       <c r="A64" s="4">
         <v>14</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>311</v>
+        <v>303</v>
       </c>
       <c r="D64" s="4" t="s">
-        <v>312</v>
+        <v>304</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>313</v>
+        <v>305</v>
       </c>
       <c r="F64" s="3" t="s">
-        <v>314</v>
+        <v>306</v>
       </c>
       <c r="G64" s="3" t="s">
-        <v>315</v>
+        <v>307</v>
       </c>
       <c r="H64" s="3" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="J64" s="3" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="65" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A65" s="4">
         <v>15</v>
       </c>
       <c r="C65" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="D65" s="4" t="s">
+        <v>309</v>
+      </c>
+      <c r="E65" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="F65" s="3" t="s">
         <v>311</v>
       </c>
-      <c r="D65" s="4" t="s">
-        <v>317</v>
-      </c>
-      <c r="E65" s="3" t="s">
-        <v>318</v>
-      </c>
-      <c r="F65" s="3" t="s">
-        <v>319</v>
-      </c>
       <c r="G65" s="3" t="s">
-        <v>320</v>
+        <v>312</v>
       </c>
       <c r="H65" s="3" t="s">
-        <v>321</v>
+        <v>313</v>
       </c>
       <c r="J65" s="3" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="66" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A66" s="4">
         <v>16</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>323</v>
+        <v>315</v>
       </c>
       <c r="D66" s="4" t="s">
-        <v>324</v>
+        <v>316</v>
       </c>
       <c r="E66" s="3" t="s">
-        <v>325</v>
+        <v>317</v>
       </c>
       <c r="F66" s="3" t="s">
-        <v>326</v>
+        <v>318</v>
       </c>
       <c r="G66" s="3" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
       <c r="H66" s="3" t="s">
-        <v>328</v>
+        <v>320</v>
       </c>
       <c r="J66" s="3" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="67" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" ht="64" x14ac:dyDescent="0.2">
       <c r="A67" s="4">
         <v>17</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>329</v>
+        <v>321</v>
       </c>
       <c r="D67" s="16" t="s">
-        <v>330</v>
+        <v>322</v>
       </c>
       <c r="E67" s="3" t="s">
-        <v>331</v>
+        <v>323</v>
       </c>
       <c r="F67" s="3" t="s">
-        <v>332</v>
+        <v>324</v>
       </c>
       <c r="G67" s="3" t="s">
-        <v>333</v>
+        <v>325</v>
       </c>
       <c r="H67" s="3" t="s">
-        <v>321</v>
+        <v>313</v>
       </c>
       <c r="J67" s="3" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="68" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A68" s="4">
         <v>18</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>334</v>
+        <v>326</v>
       </c>
       <c r="D68" s="4" t="s">
-        <v>335</v>
+        <v>327</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>336</v>
+        <v>328</v>
       </c>
       <c r="F68" s="3" t="s">
-        <v>337</v>
+        <v>329</v>
       </c>
       <c r="G68" s="3" t="s">
-        <v>338</v>
+        <v>330</v>
       </c>
       <c r="H68" s="3" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="J68" s="3" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A69" s="4">
         <v>19</v>
       </c>
       <c r="D69" s="4" t="s">
-        <v>339</v>
+        <v>331</v>
       </c>
       <c r="E69" s="3" t="s">
-        <v>340</v>
+        <v>332</v>
       </c>
       <c r="F69" s="3" t="s">
-        <v>341</v>
+        <v>333</v>
       </c>
       <c r="G69" s="3" t="s">
-        <v>342</v>
+        <v>334</v>
       </c>
       <c r="H69" s="3" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="J69" s="3" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="70" spans="1:10" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>343</v>
+        <v>335</v>
       </c>
       <c r="B70" s="11" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="C70" s="11"/>
       <c r="D70" s="11" t="s">
-        <v>344</v>
+        <v>336</v>
       </c>
       <c r="E70" t="s">
-        <v>345</v>
+        <v>337</v>
       </c>
       <c r="F70" t="s">
-        <v>346</v>
+        <v>338</v>
       </c>
       <c r="G70" t="s">
-        <v>347</v>
+        <v>339</v>
       </c>
       <c r="H70" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="I70" s="11" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="J70" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="71" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="11"/>
       <c r="B71" s="11"/>
       <c r="C71" s="11"/>
       <c r="D71" s="11"/>
     </row>
-    <row r="72" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72"/>
       <c r="B72" s="11"/>
       <c r="C72" s="11"/>
       <c r="D72" s="11"/>
     </row>
-    <row r="73" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73"/>
       <c r="B73" s="11"/>
       <c r="C73" s="11"/>
       <c r="D73" s="11"/>
     </row>
-    <row r="74" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74"/>
       <c r="B74" s="11"/>
       <c r="C74" s="11"/>
       <c r="D74" s="11"/>
     </row>
-    <row r="75" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75"/>
     </row>
   </sheetData>
@@ -4666,146 +4449,146 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{273AFAA3-99F7-4E93-9580-DCAE2B14D938}">
   <dimension ref="A1:G7"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.28515625" customWidth="1"/>
-    <col min="2" max="2" width="18.42578125" customWidth="1"/>
-    <col min="3" max="3" width="14.85546875" customWidth="1"/>
-    <col min="4" max="4" width="15.140625" customWidth="1"/>
-    <col min="5" max="5" width="16.7109375" customWidth="1"/>
-    <col min="6" max="6" width="16.42578125" customWidth="1"/>
-    <col min="7" max="7" width="41.42578125" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" customWidth="1"/>
+    <col min="2" max="2" width="18.5" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.1640625" customWidth="1"/>
+    <col min="5" max="5" width="16.6640625" customWidth="1"/>
+    <col min="6" max="6" width="16.5" customWidth="1"/>
+    <col min="7" max="7" width="41.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="195.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="195.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>343</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>346</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>349</v>
       </c>
-      <c r="B1" s="2" t="s">
+    </row>
+    <row r="3" spans="1:7" ht="64" x14ac:dyDescent="0.2">
+      <c r="C3" t="s">
+        <v>296</v>
+      </c>
+      <c r="D3" t="s">
+        <v>297</v>
+      </c>
+      <c r="E3" t="s">
+        <v>298</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="G3" t="s">
         <v>350</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+    </row>
+    <row r="4" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="C4" t="s">
         <v>351</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="D4" t="s">
         <v>352</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="E4" t="s">
+        <v>262</v>
+      </c>
+      <c r="F4" t="s">
+        <v>80</v>
+      </c>
+      <c r="G4" s="12" t="s">
         <v>353</v>
       </c>
-      <c r="D2" s="1" t="s">
+    </row>
+    <row r="5" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="C5" t="s">
         <v>354</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="D5" t="s">
         <v>355</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="E5" t="s">
+        <v>262</v>
+      </c>
+      <c r="F5" t="s">
+        <v>80</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="48" x14ac:dyDescent="0.2">
+      <c r="C6" s="11" t="s">
         <v>356</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="D6" s="11" t="s">
+        <v>280</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>281</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="G6" s="12" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+      <c r="C7" t="s">
         <v>357</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" ht="75" x14ac:dyDescent="0.25">
-      <c r="C3" t="s">
-        <v>304</v>
-      </c>
-      <c r="D3" t="s">
-        <v>305</v>
-      </c>
-      <c r="E3" t="s">
-        <v>306</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="G3" t="s">
+      <c r="D7" t="s">
         <v>358</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C4" t="s">
+      <c r="E7" t="s">
+        <v>216</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="G7" s="14" t="s">
         <v>359</v>
-      </c>
-      <c r="D4" t="s">
-        <v>360</v>
-      </c>
-      <c r="E4" t="s">
-        <v>270</v>
-      </c>
-      <c r="F4" t="s">
-        <v>88</v>
-      </c>
-      <c r="G4" s="12" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C5" t="s">
-        <v>362</v>
-      </c>
-      <c r="D5" t="s">
-        <v>363</v>
-      </c>
-      <c r="E5" t="s">
-        <v>270</v>
-      </c>
-      <c r="F5" t="s">
-        <v>88</v>
-      </c>
-      <c r="G5" s="12" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="60" x14ac:dyDescent="0.25">
-      <c r="C6" s="11" t="s">
-        <v>364</v>
-      </c>
-      <c r="D6" s="11" t="s">
-        <v>288</v>
-      </c>
-      <c r="E6" s="11" t="s">
-        <v>289</v>
-      </c>
-      <c r="F6" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="G6" s="12" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C7" t="s">
-        <v>365</v>
-      </c>
-      <c r="D7" t="s">
-        <v>366</v>
-      </c>
-      <c r="E7" t="s">
-        <v>224</v>
-      </c>
-      <c r="F7" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="G7" s="14" t="s">
-        <v>367</v>
       </c>
     </row>
   </sheetData>
@@ -4818,22 +4601,22 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2489EBC-5098-4697-9724-F190D24E1C3D}">
   <dimension ref="A1:A5"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:1" ht="111" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" ht="111" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>368</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>370</v>
+        <v>362</v>
       </c>
     </row>
   </sheetData>
@@ -4843,6 +4626,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D5656983173B1142A9B62A9C329F89A7" ma:contentTypeVersion="13" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="71caa5f225d89a4181f0614974a0635b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="bb18a1b9-ddba-4244-9634-64732d0cb267" xmlns:ns3="06294a2e-6f87-4144-83b8-94a4d04d144a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d74eef483bec37fcdf125766e7bdb283" ns2:_="" ns3:_="">
     <xsd:import namespace="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
@@ -5049,27 +4852,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E3A9028-3436-4B29-A420-9ED5B8A085B1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
+    <ds:schemaRef ds:uri="06294a2e-6f87-4144-83b8-94a4d04d144a"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148267B0-4CF5-48A7-B543-CDE45AF0A8FC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{226BE694-A00C-4E31-A532-690E39C51D9D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5086,23 +4888,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148267B0-4CF5-48A7-B543-CDE45AF0A8FC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E3A9028-3436-4B29-A420-9ED5B8A085B1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
-    <ds:schemaRef ds:uri="06294a2e-6f87-4144-83b8-94a4d04d144a"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>